<commit_message>
Added TC11, TC12, TC13, TC15
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testdata.xlsx
+++ b/src/test/resources/testData/testdata.xlsx
@@ -5,15 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497768\IdeaProjects\Hackathon-Project\src\test\resources\testData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497810\eclipse-workspace\Hackathon-Project\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B5FB2C2-B198-420E-A805-6F748AAF9F42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30950EE5-971A-467D-BDA7-BFB2E10978C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PractoData" sheetId="1" r:id="rId1"/>
+    <sheet name="HospitalTestData" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="32">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -94,13 +95,40 @@
   </si>
   <si>
     <t>TC_002</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>RequiredMatchCount</t>
+  </si>
+  <si>
+    <t>MinimumRating</t>
+  </si>
+  <si>
+    <t>TC11</t>
+  </si>
+  <si>
+    <t>TC12</t>
+  </si>
+  <si>
+    <t>TC13</t>
+  </si>
+  <si>
+    <t>TC14</t>
+  </si>
+  <si>
+    <t>TC15</t>
+  </si>
+  <si>
+    <t>hospital 24/7</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -138,8 +166,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -152,8 +193,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F5F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -161,17 +208,38 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFE6E6E6"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFE6E6E6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFE6E6E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -576,4 +644,106 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09CAE19C-3C30-4587-96DE-D311C191F8C9}">
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="2" max="2" width="23.6328125" customWidth="1"/>
+    <col min="3" max="3" width="20.08984375" customWidth="1"/>
+    <col min="4" max="4" width="27.26953125" customWidth="1"/>
+    <col min="5" max="5" width="39.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="50" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="33.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A2" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+    </row>
+    <row r="3" spans="1:5" ht="33.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="6">
+        <v>10</v>
+      </c>
+      <c r="E3" s="6">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="33.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A4" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+    </row>
+    <row r="5" spans="1:5" ht="33.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A5" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+    </row>
+    <row r="6" spans="1:5" ht="33.5" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A6" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Abinaya all testcases passed
</commit_message>
<xml_diff>
--- a/src/test/resources/testData/testdata.xlsx
+++ b/src/test/resources/testData/testdata.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2497768\IdeaProjects\Hackathon-Project\src\test\resources\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27FF9F97-B3A6-4369-9F43-238AD2BF66D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A49CF92-128B-4DAD-8A8B-0D29610B2032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PractoData" sheetId="1" r:id="rId1"/>
-    <sheet name="HospitalTestData" sheetId="2" r:id="rId2"/>
-    <sheet name="MedicineData" sheetId="3" r:id="rId3"/>
+    <sheet name="CitySearch" sheetId="4" r:id="rId2"/>
+    <sheet name="HospitalTestData" sheetId="2" r:id="rId3"/>
+    <sheet name="MedicineData" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="38">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -135,6 +136,12 @@
   </si>
   <si>
     <t>TC_018</t>
+  </si>
+  <si>
+    <t>TC_008</t>
+  </si>
+  <si>
+    <t>CityName</t>
   </si>
 </sst>
 </file>
@@ -688,6 +695,35 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1463F736-355C-4F92-93B0-AF89C4FB4BBE}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09CAE19C-3C30-4587-96DE-D311C191F8C9}">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -793,7 +829,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE4B8614-B6CB-4959-8F28-25784C056AAF}">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>